<commit_message>
Modified Excel in Tutorialninja
</commit_message>
<xml_diff>
--- a/DataDriven/TutuorialNinja/Excel/Book1.xlsx
+++ b/DataDriven/TutuorialNinja/Excel/Book1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\python selenium-D\PY_pytest\TutuorialNinja_DataDriven\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5caedeb557de9d3a/Documents/Expleo training/python/Pytest/DataDriven/TutuorialNinja/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70165040-6190-428F-B669-A4C5CF6F400A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{70165040-6190-428F-B669-A4C5CF6F400A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1E8108B-CE90-49B9-8E5E-B4CC189D12E9}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2385" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{04688EDC-C1A9-40DB-8040-96C96F39DAF7}"/>
+    <workbookView xWindow="1392" yWindow="3720" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{04688EDC-C1A9-40DB-8040-96C96F39DAF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,14 +35,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>userName</t>
   </si>
   <si>
-    <t>aakash88@gmail.com</t>
-  </si>
-  <si>
     <t>password</t>
   </si>
   <si>
@@ -53,6 +50,12 @@
   </si>
   <si>
     <t>canon</t>
+  </si>
+  <si>
+    <t>mythily@gmail.com</t>
+  </si>
+  <si>
+    <t>mythily</t>
   </si>
 </sst>
 </file>
@@ -416,22 +419,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EED7838F-3C8D-4C06-A369-F8FE593B29F1}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.21875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -445,21 +451,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A9BD7BB-CD18-4E24-AEFC-9FD4310523B9}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>